<commit_message>
final push of v2.0
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,29 +469,44 @@
           <t>payment_date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>utr</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>course</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>mark</t>
+          <t>valli</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>markmession001@gmail.com</t>
+          <t>suresh2004krishna@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>vsv clg</t>
+          <t>tce</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>8111005543</t>
+          <t>07904900115</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -500,17 +515,32 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>499</v>
+        <v>299</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06-06-2026</t>
+          <t>10-06-2026 12:35</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>784512369874</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2nd Year</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Python Programming</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -519,12 +549,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>suresh2004krishna@gmail.com</t>
+          <t>sureh2004krishna@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>tce</t>
+          <t>gov school</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -534,47 +564,32 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Pending Verification</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>499</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ram</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>suresh2004krishna@gmail.com</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>mmc clg</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>07904900115</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>499</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
+        <v>299</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>10-06-2026 16:02</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>12345678790115</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Higher Secondary</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Python Programming</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>